<commit_message>
renomeia paginas para menu lateral APS mais elegante
</commit_message>
<xml_diff>
--- a/OEE - 2026.xlsx
+++ b/OEE - 2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBB24F4-3273-44BB-A4E8-F4444F28A7BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D514ECA-A3B0-4041-8250-8423BC4CF739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C4D301CD-4AF9-4F8B-9B61-A5A68A12AAB1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>MÊS</t>
   </si>
@@ -84,6 +84,15 @@
   </si>
   <si>
     <t>PEÇAS REFUGADAS</t>
+  </si>
+  <si>
+    <t>DISPONIBILIDADE (H)</t>
+  </si>
+  <si>
+    <t>PARADAS DE MAQUINA (H)</t>
+  </si>
+  <si>
+    <t>TEMPO OPERANDO (H)</t>
   </si>
 </sst>
 </file>
@@ -92,7 +101,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -166,15 +175,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -510,15 +520,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E445367D-2B9F-4C32-869A-9253C4DC7A76}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="35.88671875" customWidth="1"/>
-    <col min="3" max="3" width="32.21875" customWidth="1"/>
-    <col min="4" max="4" width="34.44140625" customWidth="1"/>
+    <col min="2" max="2" width="38.44140625" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" customWidth="1"/>
+    <col min="6" max="6" width="23.77734375" customWidth="1"/>
+    <col min="7" max="7" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -531,8 +544,17 @@
       <c r="D1" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -545,8 +567,19 @@
       <c r="D2" s="1">
         <v>142</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" s="4">
+        <f>12*220</f>
+        <v>2640</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <f>(E2-F2)*0.8</f>
+        <v>2112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -559,8 +592,19 @@
       <c r="D3" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" s="4">
+        <f t="shared" ref="E3:E4" si="0">12*220</f>
+        <v>2640</v>
+      </c>
+      <c r="F3" s="4">
+        <v>36</v>
+      </c>
+      <c r="G3" s="4">
+        <f t="shared" ref="G3:G4" si="1">(E3-F3)*0.8</f>
+        <v>2083.2000000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -574,78 +618,116 @@
       <c r="D4" s="1">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4" s="4">
+        <f t="shared" si="0"/>
+        <v>2640</v>
+      </c>
+      <c r="F4" s="4">
+        <v>98</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" si="1"/>
+        <v>2033.6000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
atualiza OEE - 2026.xlsx
</commit_message>
<xml_diff>
--- a/OEE - 2026.xlsx
+++ b/OEE - 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D514ECA-A3B0-4041-8250-8423BC4CF739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE5B921-3654-48D6-9FBA-65417104A5CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C4D301CD-4AF9-4F8B-9B61-A5A68A12AAB1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -175,7 +175,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -185,6 +185,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -519,15 +520,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E445367D-2B9F-4C32-869A-9253C4DC7A76}">
-  <dimension ref="A1:G13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="38.44140625" customWidth="1"/>
     <col min="3" max="3" width="36" customWidth="1"/>
     <col min="4" max="4" width="25.6640625" customWidth="1"/>
     <col min="5" max="5" width="21.6640625" customWidth="1"/>
-    <col min="6" max="6" width="23.77734375" customWidth="1"/>
+    <col min="6" max="6" width="25.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -593,14 +594,14 @@
         <v>0</v>
       </c>
       <c r="E3" s="4">
-        <f t="shared" ref="E3:E4" si="0">12*220</f>
+        <f t="shared" ref="E3" si="0">12*220</f>
         <v>2640</v>
       </c>
       <c r="F3" s="4">
         <v>36</v>
       </c>
       <c r="G3" s="4">
-        <f t="shared" ref="G3:G4" si="1">(E3-F3)*0.8</f>
+        <f t="shared" ref="G3:G5" si="1">(E3-F3)*0.8</f>
         <v>2083.2000000000003</v>
       </c>
     </row>
@@ -619,7 +620,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="4">
-        <f t="shared" si="0"/>
+        <f>12*220</f>
         <v>2640</v>
       </c>
       <c r="F4" s="4">
@@ -634,12 +635,26 @@
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
+      <c r="B5" s="1">
+        <v>2257</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2161</v>
+      </c>
+      <c r="D5" s="1">
+        <v>25</v>
+      </c>
+      <c r="E5" s="4">
+        <f>12*220</f>
+        <v>2640</v>
+      </c>
+      <c r="F5" s="4">
+        <v>30</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="1"/>
+        <v>2088</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
@@ -729,8 +744,17 @@
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
     </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
cleanup: remove marcadores visuais e logs temporarios da APS
</commit_message>
<xml_diff>
--- a/OEE - 2026.xlsx
+++ b/OEE - 2026.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manutencao\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE5B921-3654-48D6-9FBA-65417104A5CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4575"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -98,12 +97,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -520,19 +519,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="38.44140625" customWidth="1"/>
+    <col min="2" max="2" width="38.5" customWidth="1"/>
     <col min="3" max="3" width="36" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" customWidth="1"/>
-    <col min="6" max="6" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.109375" customWidth="1"/>
+    <col min="4" max="4" width="25.625" customWidth="1"/>
+    <col min="5" max="5" width="21.625" customWidth="1"/>
+    <col min="6" max="6" width="25.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -555,7 +554,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="15">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -580,7 +579,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="15">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -601,11 +600,11 @@
         <v>36</v>
       </c>
       <c r="G3" s="4">
-        <f t="shared" ref="G3:G5" si="1">(E3-F3)*0.8</f>
+        <f t="shared" ref="G3:G6" si="1">(E3-F3)*0.8</f>
         <v>2083.2000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="15">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -631,7 +630,7 @@
         <v>2033.6000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="15">
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
@@ -656,18 +655,28 @@
         <v>2088</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="15">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D6" s="1">
+        <v>24</v>
+      </c>
+      <c r="E6" s="4">
+        <f>12*220</f>
+        <v>2640</v>
+      </c>
+      <c r="F6" s="4">
+        <v>157</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="1"/>
+        <v>1986.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -678,7 +687,7 @@
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="15">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -689,7 +698,7 @@
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="15">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
@@ -700,7 +709,7 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="15">
       <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
@@ -711,7 +720,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="15">
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
@@ -722,7 +731,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="15">
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
@@ -733,7 +742,7 @@
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="15">
       <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
@@ -744,11 +753,11 @@
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7">
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7">
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
     </row>

</xml_diff>

<commit_message>
atualiza PV.xlsx e outros arquivos .xlsx
</commit_message>
<xml_diff>
--- a/OEE - 2026.xlsx
+++ b/OEE - 2026.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manutencao\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_9AD4325B7883644077149C63DEF12EE8BD99EF3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4575"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -97,12 +98,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -519,19 +520,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="38.5" customWidth="1"/>
+    <col min="2" max="2" width="38.44140625" customWidth="1"/>
     <col min="3" max="3" width="36" customWidth="1"/>
-    <col min="4" max="4" width="25.625" customWidth="1"/>
-    <col min="5" max="5" width="21.625" customWidth="1"/>
-    <col min="6" max="6" width="25.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.125" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" customWidth="1"/>
+    <col min="6" max="6" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -554,7 +555,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -579,7 +580,7 @@
         <v>2112</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -604,7 +605,7 @@
         <v>2083.2000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -630,7 +631,7 @@
         <v>2033.6000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
@@ -655,7 +656,7 @@
         <v>2088</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
@@ -676,7 +677,7 @@
         <v>1986.4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -687,7 +688,7 @@
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" ht="15">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -698,7 +699,7 @@
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:7" ht="15">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
@@ -709,7 +710,7 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" ht="15">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
@@ -720,7 +721,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:7" ht="15">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
@@ -731,7 +732,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:7" ht="15">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
@@ -742,7 +743,7 @@
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:7" ht="15">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
@@ -753,11 +754,11 @@
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
     </row>

</xml_diff>